<commit_message>
[docs]update readme for V2.0
</commit_message>
<xml_diff>
--- a/docs/hardware_config/hardware.xlsx
+++ b/docs/hardware_config/hardware.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Git_doc\Real-Time-Embedded-Programming\docs\hardware_config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4130154-B28E-48E0-913B-EDCA93238B13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA7C489C-C205-4417-A24F-6417BEBF102E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{63C2FDA4-BCDA-4139-88D7-DB170DFC6997}"/>
   </bookViews>
@@ -248,6 +248,2143 @@
         </a:extLst>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>365125</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>396875</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="65" name="矩形 64">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7091F9ED-4E02-618D-BC66-3476DA691EA0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5699125" y="555625"/>
+          <a:ext cx="24701500" cy="11906250"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg1"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>249972</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>146631</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>53</xdr:col>
+      <xdr:colOff>662145</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>98140</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="图片 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C392E97F-92FB-B5EE-C0BA-692CB21C31CF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="29221992" y="5020111"/>
+          <a:ext cx="7809634" cy="5746173"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>259354</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>172358</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>544288</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>154217</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="图片 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{45FCDB5D-8D1E-032D-1F11-8E4221F8FC12}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="26704" t="13888" r="44428"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="5400000">
+          <a:off x="18104712" y="515214"/>
+          <a:ext cx="2340431" cy="4920434"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>509732</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>136813</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>416214</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>116031</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="图片 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6A6AD6B2-2DD8-8E6F-B760-721F75C7ADF6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="16648546" y="4745181"/>
+          <a:ext cx="7772400" cy="5829300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>415636</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>69273</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>623454</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>150090</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="矩形 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDD56BB3-27D7-69AE-9940-5CFC0C966062}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="20816454" y="8035637"/>
+          <a:ext cx="865909" cy="1119908"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>107949</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>120650</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>577272</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="矩形 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C887E335-4CF8-49A1-9DD8-ACF91D58B689}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21166858" y="4796559"/>
+          <a:ext cx="469323" cy="2604077"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>314037</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>23091</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>23091</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>80818</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="矩形 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87416BC3-3C1E-4159-A2F1-540DAD91993C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18740582" y="6777182"/>
+          <a:ext cx="1025236" cy="750454"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>186169</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>150090</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>555624</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>48347</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="12" name="连接符: 肘形 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{51E95805-5CFF-8807-920A-9D01D60F6324}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="6" idx="2"/>
+          <a:endCxn id="13" idx="1"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="16200000" flipH="1">
+          <a:off x="21321206" y="9431553"/>
+          <a:ext cx="771382" cy="369455"/>
+        </a:xfrm>
+        <a:prstGeom prst="bentConnector2">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>555625</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>80818</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>285750</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>15876</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="文本框 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B874F382-54E8-1BF8-4DD2-501956A6BE9D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21891625" y="9510568"/>
+          <a:ext cx="1730375" cy="982808"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="2000"/>
+            <a:t>2.Microphone</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="2000"/>
+            <a:t>Speaker</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="2000"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>11544</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>138546</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>631790</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>103909</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="24" name="图片 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{73416135-4A56-83E3-C1DA-BF798DCCDDC3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22386635" y="3775364"/>
+          <a:ext cx="5226882" cy="4641272"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>577272</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>34636</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>11544</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>37234</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="25" name="连接符: 肘形 24">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{944D3DD0-485C-4CDF-B8A6-D9E1CEEA1772}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="9" idx="3"/>
+          <a:endCxn id="24" idx="1"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="21636181" y="6096000"/>
+          <a:ext cx="750454" cy="2598"/>
+        </a:xfrm>
+        <a:prstGeom prst="bentConnector3">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 50000"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>375803</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>46182</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>34636</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>103909</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="30" name="矩形 29">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2134B09E-C17A-42B7-A877-B2AA4A2E25BA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="24725167" y="3856182"/>
+          <a:ext cx="316924" cy="750454"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>8657</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>60037</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>265545</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>103909</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="31" name="矩形 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1661428F-2B50-4469-950D-3E84D39D2781}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25016112" y="4389582"/>
+          <a:ext cx="256888" cy="217054"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>635001</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>109682</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>534266</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>46182</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="32" name="连接符: 肘形 31">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E001A421-C7C4-48C8-B058-71DBF4BC4B72}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="30" idx="0"/>
+          <a:endCxn id="43" idx="3"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="16200000" flipV="1">
+          <a:off x="22558520" y="1531072"/>
+          <a:ext cx="802409" cy="3847811"/>
+        </a:xfrm>
+        <a:prstGeom prst="bentConnector2">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>82170</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>38875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>624229</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>153175</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="40" name="图片 39">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B8322E9-276A-45F3-F511-FC865AFDFB22}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6082920" y="4404500"/>
+          <a:ext cx="7876309" cy="5876925"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>415636</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>13854</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>39</xdr:col>
+      <xdr:colOff>129309</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>115455</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="41" name="文本框 40">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1480CFC9-54DC-4F83-A7D9-D1F793D0DBB1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22790727" y="1052945"/>
+          <a:ext cx="3004127" cy="1660237"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>Rpi</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>(pin1) -&gt; PCB9865(VCC)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>Rpi(pin3) -&gt; PCB9865(SDA)</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="zh-CN" sz="1600">
+            <a:effectLst/>
+            <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>Rpi(pin5) -&gt; PCB9865(SCL)</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="zh-CN" sz="1600">
+            <a:effectLst/>
+            <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>Rpi(pin6) -&gt; PCB9865(GND)</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>648855</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>161637</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>635000</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>57727</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="43" name="矩形 42">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{253D465C-BEB2-40FF-8C06-127E25CD9C53}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="20391582" y="2586182"/>
+          <a:ext cx="644236" cy="935181"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>221961</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>51954</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>314037</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>152399</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="50" name="连接符: 肘形 49">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{02F2A68F-65C7-426D-8DAF-380F60520D12}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="10" idx="1"/>
+          <a:endCxn id="53" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="10800000" flipV="1">
+          <a:off x="18890961" y="7211579"/>
+          <a:ext cx="92076" cy="2195945"/>
+        </a:xfrm>
+        <a:prstGeom prst="bentConnector2">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>94672</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>349250</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="53" name="文本框 52">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0023421B-D847-4782-8E8A-5C6E6368A5E0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18096922" y="9407525"/>
+          <a:ext cx="1588078" cy="1038225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="2000"/>
+            <a:t>1.Screen</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="2000"/>
+            <a:t>Camera</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="2000"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>145143</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>64326</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>565726</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>172358</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="57" name="矩形 56">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DFD43D18-4A6B-4E32-8F61-280E865688A1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18024929" y="1878612"/>
+          <a:ext cx="420583" cy="833746"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>179615</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>17156</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>600198</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>125187</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="58" name="矩形 57">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8DC4FFB8-9601-4C4E-A632-B4FAD0424094}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18721615" y="2012870"/>
+          <a:ext cx="420583" cy="833746"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>168730</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>69770</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>589313</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>177801</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="59" name="矩形 58">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EC30A857-733C-4511-8F81-6DE7512ECEB0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19372944" y="2065484"/>
+          <a:ext cx="420583" cy="833746"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>21772</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>140527</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>442355</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>67130</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="60" name="矩形 59">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C4156145-EB99-4A74-B3F4-4C134908C6FB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19888201" y="2136241"/>
+          <a:ext cx="420583" cy="833746"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>290285</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>117928</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>117929</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>27215</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="61" name="文本框 60">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B2A76B7C-62A7-4953-8BAD-5ABE1E4D6344}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13534571" y="1206499"/>
+          <a:ext cx="3138715" cy="1905002"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600"/>
+            <a:t>Channel 15:Base</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600" baseline="0"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600"/>
+            <a:t>(MG996R)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600"/>
+            <a:t>Channel 11:Shoulder (MG996R)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600"/>
+            <a:t>Channel 7:Elbow (MG996R)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600"/>
+            <a:t>Channel 3:Hand (MG90S)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600"/>
+            <a:t>see more</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600" baseline="0"/>
+            <a:t> detile in include/common/servo_config.txt</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1600"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>483054</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>84737</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>238125</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>15875</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="66" name="矩形 65">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2E006947-0FD7-44D8-B1AC-ED31FDAE4055}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12484554" y="8117487"/>
+          <a:ext cx="1088571" cy="978888"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>540204</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>110137</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>295275</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>41275</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="67" name="矩形 66">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A5B368AE-E897-4B39-B889-DD8A01007017}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11874954" y="6920512"/>
+          <a:ext cx="1088571" cy="978888"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>120196</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>-1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>614590</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>83911</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="69" name="文本框 68">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{737E7C61-3278-495E-ABCB-5D09D165ECBF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14121946" y="7159624"/>
+          <a:ext cx="3161394" cy="1830162"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600"/>
+            <a:t>Servo</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600" baseline="0"/>
+            <a:t>        PCB9685</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600" baseline="0"/>
+            <a:t>BROWN        GND</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600" baseline="0"/>
+            <a:t>RED              +V</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1600" baseline="0"/>
+            <a:t>YELLOW        PWM</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>295275</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>-1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>367393</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>75706</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="70" name="连接符: 肘形 69">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C89D5EC0-8956-43D7-AC0D-88AF19AFAB6A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="67" idx="3"/>
+          <a:endCxn id="69" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="12963525" y="7159624"/>
+          <a:ext cx="2739118" cy="250332"/>
+        </a:xfrm>
+        <a:prstGeom prst="bentConnector4">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 21146"/>
+            <a:gd name="adj2" fmla="val 286837"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>360589</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>83911</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>367392</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>15875</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="74" name="连接符: 肘形 73">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5200A336-C5EA-4A95-8460-CBDD7330759F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="66" idx="2"/>
+          <a:endCxn id="69" idx="2"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="5400000" flipH="1" flipV="1">
+          <a:off x="14312446" y="7706179"/>
+          <a:ext cx="106589" cy="2673803"/>
+        </a:xfrm>
+        <a:prstGeom prst="bentConnector3">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -214469"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>88900</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>555625</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>9526</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="82" name="文本框 81">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B2BC91A6-69C1-48E7-A6E9-B48721FCC036}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19424650" y="3937000"/>
+          <a:ext cx="1800225" cy="612776"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="2000"/>
+            <a:t>3.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="2000" baseline="0"/>
+            <a:t> Servo</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="2000"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>555625</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>52388</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>342611</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>120650</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="83" name="连接符: 肘形 82">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{17705379-730C-41AB-8298-533F9D6B714F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="82" idx="3"/>
+          <a:endCxn id="9" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="21224875" y="4243388"/>
+          <a:ext cx="453736" cy="592137"/>
+        </a:xfrm>
+        <a:prstGeom prst="bentConnector2">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -685,5 +2822,6 @@
   <sheetData/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>